<commit_message>
feat: initialize English testing application with admin and student portals
</commit_message>
<xml_diff>
--- a/legacy/sample_questions_template.xlsx
+++ b/legacy/sample_questions_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\EnglishTools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\EnglishTools\legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="95">
   <si>
     <t>question_id</t>
   </si>
@@ -209,36 +209,6 @@
   </si>
   <si>
     <t>syntax</t>
-  </si>
-  <si>
-    <t>Q7</t>
-  </si>
-  <si>
-    <t>short_answer</t>
-  </si>
-  <si>
-    <t>Write an essay about water</t>
-  </si>
-  <si>
-    <t>Teacher will grade manually</t>
-  </si>
-  <si>
-    <t>writing</t>
-  </si>
-  <si>
-    <t>Q8</t>
-  </si>
-  <si>
-    <t>matching</t>
-  </si>
-  <si>
-    <t>Match pairs (Cat:Meow, Dog:Bark)</t>
-  </si>
-  <si>
-    <t>{"Cat":"Meow", "Dog":"Bark"}</t>
-  </si>
-  <si>
-    <t>Animal sounds</t>
   </si>
   <si>
     <t>Column</t>
@@ -687,7 +657,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="15" width="18" customWidth="1"/>
@@ -745,7 +715,7 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C2" t="s">
         <v>17</v>
@@ -792,7 +762,7 @@
         <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
         <v>29</v>
@@ -836,7 +806,7 @@
         <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
         <v>35</v>
@@ -874,7 +844,7 @@
         <v>41</v>
       </c>
       <c r="B5" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C5" t="s">
         <v>42</v>
@@ -918,7 +888,7 @@
         <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C6" t="s">
         <v>51</v>
@@ -953,7 +923,7 @@
         <v>57</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
         <v>58</v>
@@ -977,67 +947,6 @@
         <v>62</v>
       </c>
       <c r="O7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B8" t="s">
-        <v>104</v>
-      </c>
-      <c r="C8" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E8" t="s">
-        <v>65</v>
-      </c>
-      <c r="L8" t="s">
-        <v>66</v>
-      </c>
-      <c r="M8">
-        <v>10</v>
-      </c>
-      <c r="N8" t="s">
-        <v>67</v>
-      </c>
-      <c r="O8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" t="s">
-        <v>70</v>
-      </c>
-      <c r="K9" t="s">
-        <v>71</v>
-      </c>
-      <c r="L9" t="s">
-        <v>72</v>
-      </c>
-      <c r="M9">
-        <v>5</v>
-      </c>
-      <c r="N9" t="s">
-        <v>49</v>
-      </c>
-      <c r="O9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1059,16 +968,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1076,13 +985,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1090,10 +999,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="D3" t="s">
         <v>16</v>
@@ -1104,13 +1013,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="D4" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1118,13 +1027,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1132,27 +1041,27 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="D6" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B7" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D7" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1160,13 +1069,13 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1174,13 +1083,13 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -1188,13 +1097,13 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="C10" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="D10" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -1202,13 +1111,13 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C11" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="D11" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -1216,13 +1125,13 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="D12" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -1230,13 +1139,13 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="C13" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="D13" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>